<commit_message>
feat: add opitdev pre-corte analyzer to hub
</commit_message>
<xml_diff>
--- a/input/repositorios_github_pages.xlsx
+++ b/input/repositorios_github_pages.xlsx
@@ -372,7 +372,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43.5703125" customWidth="1" min="1" max="1"/>
@@ -641,6 +641,28 @@
       <c r="D12" s="3" t="inlineStr">
         <is>
           <t>https://silvathiagoferreira.github.io/plano-de-fogo-previsto/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>analizador-de-pre-corte-opitdev</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>ANALIZADOR DE PRÉ-CORTE - OPITDEV</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/SILVAThiagoFerreira/analizador-de-pre-corte-opitdev</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>https://silvathiagoferreira.github.io/analizador-de-pre-corte-opitdev/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(hub): adicionar atalho para aviso de desmonte
</commit_message>
<xml_diff>
--- a/input/repositorios_github_pages.xlsx
+++ b/input/repositorios_github_pages.xlsx
@@ -372,7 +372,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43.5703125" customWidth="1" min="1" max="1"/>
@@ -663,6 +663,28 @@
       <c r="D13" s="3" t="inlineStr">
         <is>
           <t>https://silvathiagoferreira.github.io/analizador-de-pre-corte-opitdev/</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>aviso-desmonte</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Criador de Aviso de Desmonte</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/SILVAThiagoFerreira/aviso-desmonte</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>https://silvathiagoferreira.github.io/aviso-desmonte/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add depth report to US Vale Verde hub
</commit_message>
<xml_diff>
--- a/input/repositorios_github_pages.xlsx
+++ b/input/repositorios_github_pages.xlsx
@@ -372,7 +372,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43.5703125" customWidth="1" min="1" max="1"/>
@@ -685,6 +685,28 @@
       <c r="D14" t="inlineStr">
         <is>
           <t>https://silvathiagoferreira.github.io/planejador-campanha-sismografia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>relatorio-profundidades-opitdev</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Relatório de Profundidades - OPITDEV</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>https://github.com/SILVAThiagoFerreira/relatorio-profundidades-opitdev</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://silvathiagoferreira.github.io/relatorio-profundidades-opitdev/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adiciona ferramenta CHI ao hub US Vale Verde
</commit_message>
<xml_diff>
--- a/input/repositorios_github_pages.xlsx
+++ b/input/repositorios_github_pages.xlsx
@@ -372,7 +372,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43.5703125" customWidth="1" min="1" max="1"/>
@@ -707,6 +707,28 @@
       <c r="D15" t="inlineStr">
         <is>
           <t>https://silvathiagoferreira.github.io/relatorio-profundidades-opitdev/</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>chi-usvaleverde</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Carteira de Habilitação Interna - CHI - Enaex Brasil</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>https://github.com/SILVAThiagoFerreira/chi-usvaleverde</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://silvathiagoferreira.github.io/chi-usvaleverde/</t>
         </is>
       </c>
     </row>

</xml_diff>